<commit_message>
Fix photo import and header text wrapping
- Photo path resolution: try relative, basename-only, and absolute paths
- Handle backslashes in Windows photo paths
- Add more photo column aliases
- Fix header title wrapping by reducing font to 13.5pt + nowrap

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sample/test_students.xlsx
+++ b/sample/test_students.xlsx
@@ -1,17 +1,50 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+  <workbookPr/>
+  <bookViews>
+    <workbookView windowWidth="20490" windowHeight="7845"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Students" state="visible" r:id="rId4"/>
+    <sheet name="Students" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <calcPr calcId="144525"/>
 </workbook>
 </file>
 
+<file path=xl/cellimages.xml><?xml version="1.0" encoding="utf-8"?>
+<etc:cellImages xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <etc:cellImage>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="ID_5367125F7A534A478B711DB5F9F4C130" descr="Pi7_Passport_Photo (5)"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9439275" y="200025"/>
+          <a:ext cx="3933825" cy="5057775"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+  </etc:cellImage>
+</etc:cellImages>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="42">
   <si>
     <t>Symbol No</t>
   </si>
@@ -82,34 +115,34 @@
     <t>Account</t>
   </si>
   <si>
+    <t>1002</t>
+  </si>
+  <si>
+    <t>Sita Kumari Rai</t>
+  </si>
+  <si>
+    <t>Female</t>
+  </si>
+  <si>
+    <t>Kumar Rai</t>
+  </si>
+  <si>
+    <t>2068/08/22</t>
+  </si>
+  <si>
+    <t>Everest Academy</t>
+  </si>
+  <si>
+    <t>Dharan-5, Sunsari</t>
+  </si>
+  <si>
+    <t>9823456789</t>
+  </si>
+  <si>
+    <t>sita@test.com</t>
+  </si>
+  <si>
     <t/>
-  </si>
-  <si>
-    <t>1002</t>
-  </si>
-  <si>
-    <t>Sita Kumari Rai</t>
-  </si>
-  <si>
-    <t>Female</t>
-  </si>
-  <si>
-    <t>Kumar Rai</t>
-  </si>
-  <si>
-    <t>2068/08/22</t>
-  </si>
-  <si>
-    <t>Everest Academy</t>
-  </si>
-  <si>
-    <t>Dharan-5, Sunsari</t>
-  </si>
-  <si>
-    <t>9823456789</t>
-  </si>
-  <si>
-    <t>sita@test.com</t>
   </si>
   <si>
     <t>1003</t>
@@ -142,25 +175,368 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
-    <font>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="4">
+    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
+  </numFmts>
+  <fonts count="21">
+    <font>
+      <sz val="11"/>
       <color theme="1"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="33">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -168,24 +544,310 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="4" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="11" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="19" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
   <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="60% - Accent6" xfId="1" builtinId="52"/>
+    <cellStyle name="40% - Accent6" xfId="2" builtinId="51"/>
+    <cellStyle name="60% - Accent5" xfId="3" builtinId="48"/>
+    <cellStyle name="Accent6" xfId="4" builtinId="49"/>
+    <cellStyle name="40% - Accent5" xfId="5" builtinId="47"/>
+    <cellStyle name="20% - Accent5" xfId="6" builtinId="46"/>
+    <cellStyle name="60% - Accent4" xfId="7" builtinId="44"/>
+    <cellStyle name="Accent5" xfId="8" builtinId="45"/>
+    <cellStyle name="40% - Accent4" xfId="9" builtinId="43"/>
+    <cellStyle name="Accent4" xfId="10" builtinId="41"/>
+    <cellStyle name="Linked Cell" xfId="11" builtinId="24"/>
+    <cellStyle name="40% - Accent3" xfId="12" builtinId="39"/>
+    <cellStyle name="60% - Accent2" xfId="13" builtinId="36"/>
+    <cellStyle name="Accent3" xfId="14" builtinId="37"/>
+    <cellStyle name="40% - Accent2" xfId="15" builtinId="35"/>
+    <cellStyle name="20% - Accent2" xfId="16" builtinId="34"/>
+    <cellStyle name="Accent2" xfId="17" builtinId="33"/>
+    <cellStyle name="40% - Accent1" xfId="18" builtinId="31"/>
+    <cellStyle name="20% - Accent1" xfId="19" builtinId="30"/>
+    <cellStyle name="Accent1" xfId="20" builtinId="29"/>
+    <cellStyle name="Neutral" xfId="21" builtinId="28"/>
+    <cellStyle name="60% - Accent1" xfId="22" builtinId="32"/>
+    <cellStyle name="Bad" xfId="23" builtinId="27"/>
+    <cellStyle name="20% - Accent4" xfId="24" builtinId="42"/>
+    <cellStyle name="Total" xfId="25" builtinId="25"/>
+    <cellStyle name="Output" xfId="26" builtinId="21"/>
+    <cellStyle name="Currency" xfId="27" builtinId="4"/>
+    <cellStyle name="20% - Accent3" xfId="28" builtinId="38"/>
+    <cellStyle name="Note" xfId="29" builtinId="10"/>
+    <cellStyle name="Input" xfId="30" builtinId="20"/>
+    <cellStyle name="Heading 4" xfId="31" builtinId="19"/>
+    <cellStyle name="Calculation" xfId="32" builtinId="22"/>
+    <cellStyle name="Good" xfId="33" builtinId="26"/>
+    <cellStyle name="Heading 3" xfId="34" builtinId="18"/>
+    <cellStyle name="CExplanatory Text" xfId="35" builtinId="53"/>
+    <cellStyle name="Heading 1" xfId="36" builtinId="16"/>
+    <cellStyle name="Comma [0]" xfId="37" builtinId="6"/>
+    <cellStyle name="20% - Accent6" xfId="38" builtinId="50"/>
+    <cellStyle name="Title" xfId="39" builtinId="15"/>
+    <cellStyle name="Currency [0]" xfId="40" builtinId="7"/>
+    <cellStyle name="Warning Text" xfId="41" builtinId="11"/>
+    <cellStyle name="Followed Hyperlink" xfId="42" builtinId="9"/>
+    <cellStyle name="Heading 2" xfId="43" builtinId="17"/>
+    <cellStyle name="Comma" xfId="44" builtinId="3"/>
+    <cellStyle name="Check Cell" xfId="45" builtinId="23"/>
+    <cellStyle name="60% - Accent3" xfId="46" builtinId="40"/>
+    <cellStyle name="Percent" xfId="47" builtinId="5"/>
+    <cellStyle name="Hyperlink" xfId="48" builtinId="8"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -507,16 +1169,16 @@
       </a:style>
     </a:lnDef>
   </a:objectDefaults>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:L4"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelRow="3"/>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -554,7 +1216,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="2" ht="75" spans="1:12">
       <c r="A2" t="s">
         <v>12</v>
       </c>
@@ -588,37 +1250,38 @@
       <c r="K2" t="s">
         <v>22</v>
       </c>
-      <c r="L2" t="s">
+      <c r="L2" t="str">
+        <f>_xlfn.DISPIMG("ID_5367125F7A534A478B711DB5F9F4C130",1)</f>
+        <v>=DISPIMG("ID_5367125F7A534A478B711DB5F9F4C130",1)</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12">
+      <c r="A3" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="B3" t="s">
         <v>24</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
         <v>25</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>26</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>27</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>28</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>29</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>30</v>
       </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
         <v>31</v>
-      </c>
-      <c r="I3" t="s">
-        <v>32</v>
       </c>
       <c r="J3" t="s">
         <v>21</v>
@@ -627,10 +1290,10 @@
         <v>22</v>
       </c>
       <c r="L3" t="s">
-        <v>23</v>
+        <v>32</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12">
       <c r="A4" t="s">
         <v>33</v>
       </c>
@@ -665,11 +1328,12 @@
         <v>22</v>
       </c>
       <c r="L4" t="s">
-        <v>23</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup paperSize="1" orientation="portrait"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>